<commit_message>
📊 Weekly RSI Screener Report – 2026-08-29
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>328</v>
+        <v>5169.2</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.53</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.17</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.01000000000001</v>
+        <v>69.19</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>38.8</v>
+        <v>50.87</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>277.7</v>
+        <v>4439.24</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>276.21</v>
+        <v>4323.1</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>31386238</v>
+        <v>811562</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>301937</v>
+        <v>458669</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>5086.1</v>
+        <v>328</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.13</v>
+        <v>65.69</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>72.23</v>
+        <v>68.17</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>68.48</v>
+        <v>66.01000000000001</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>52.06</v>
+        <v>41.27</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>4392.15</v>
+        <v>280.96</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>4282.33</v>
+        <v>278.71</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>851335</v>
+        <v>31526889</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>451296</v>
+        <v>301937</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,31 +624,31 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8042</v>
+        <v>1337.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>63.22</v>
+        <v>64.53</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>64.06</v>
+        <v>64.87</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>69.17</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>34.96</v>
+        <v>31.46</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>7304.81</v>
+        <v>1236.47</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>7153.89</v>
+        <v>1216.25</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>495308</v>
+        <v>1804528</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>219892</v>
+        <v>325846</v>
       </c>
     </row>
     <row r="5">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11700</v>
+        <v>11910</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>62.91</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>73.20999999999999</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.02</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>54.07</v>
+        <v>52.36</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>10186.02</v>
+        <v>10292.1</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>9960.559999999999</v>
+        <v>10056.1</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>410254</v>
+        <v>341405</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>321256</v>
+        <v>327022</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,31 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1130</v>
+        <v>8059</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>60.96</v>
+        <v>60.94</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>65.7</v>
+        <v>64.83</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>71.39</v>
+        <v>69.45999999999999</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>21.38</v>
+        <v>35.22</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>986.88</v>
+        <v>7362.25</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>954.4</v>
+        <v>7206.37</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5018614</v>
+        <v>436761</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>265883</v>
+        <v>221237</v>
       </c>
     </row>
     <row r="7">
@@ -741,70 +741,31 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3308</v>
+        <v>3258</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>59.7</v>
+        <v>52.57</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>65.93000000000001</v>
+        <v>64.61</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>68.13</v>
+        <v>67.8</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>25.83</v>
+        <v>25.33</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>3007.1</v>
+        <v>3021.5</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>2959.36</v>
+        <v>2972.27</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>804541</v>
+        <v>880922</v>
       </c>
       <c r="K7" s="4" t="n">
-        <v>224366</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>APOLLOHOSP</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>8693</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>45.18</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>61.69</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>65.86</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>21.97</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>8206.190000000001</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>8048.12</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>356988</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>124992</v>
+        <v>223145</v>
       </c>
     </row>
   </sheetData>
@@ -815,7 +776,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -873,7 +833,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -882,16 +842,16 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>328</v>
+        <v>423.7</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>69.53</v>
+        <v>74.16</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.17</v>
+        <v>61.93</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.01000000000001</v>
+        <v>56.77</v>
       </c>
     </row>
     <row r="3">
@@ -906,22 +866,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>5086.1</v>
+        <v>5169.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>69.13</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>72.23</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>68.48</v>
+        <v>69.19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -930,22 +890,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>8042</v>
+        <v>3168.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>63.22</v>
+        <v>66.52</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>64.06</v>
+        <v>67.81</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>69.17</v>
+        <v>60.73</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -954,22 +914,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11700</v>
+        <v>328</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>62.91</v>
+        <v>65.69</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>73.20999999999999</v>
+        <v>68.17</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.02</v>
+        <v>66.01000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -978,22 +938,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>402.8</v>
+        <v>1337.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>62.21</v>
+        <v>64.53</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>54.56</v>
+        <v>64.87</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>52.93</v>
+        <v>67.06999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1002,22 +962,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>2032.5</v>
+        <v>11910</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>61.18</v>
+        <v>64.43000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>61.08</v>
+        <v>74.95999999999999</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>57.64</v>
+        <v>68.81999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1026,22 +986,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1130</v>
+        <v>1640.9</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>60.96</v>
+        <v>61.51</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>65.7</v>
+        <v>61.97</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>71.39</v>
+        <v>58.68</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1050,22 +1010,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>414</v>
+        <v>8059</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>60.83</v>
+        <v>60.94</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>50.12</v>
+        <v>64.83</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>60.32</v>
+        <v>69.45999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1074,22 +1034,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>4093</v>
+        <v>411.9</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>60.35</v>
+        <v>55.51</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>55.41</v>
+        <v>49.37</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>58.49</v>
+        <v>60.06</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1098,22 +1058,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>3308</v>
+        <v>1265</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>59.7</v>
+        <v>54.95</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>65.93000000000001</v>
+        <v>48.57</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>68.13</v>
+        <v>54.58</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1122,22 +1082,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>3412.2</v>
+        <v>2002</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>57.13</v>
+        <v>53.65</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>57.93</v>
+        <v>58.37</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>62.11</v>
+        <v>56.37</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1146,22 +1106,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1293.7</v>
+        <v>2342</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>55.95</v>
+        <v>53.64</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>59.84</v>
+        <v>47.46</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>65.2</v>
+        <v>38.69</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1170,22 +1130,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1095</v>
+        <v>1037.4</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>55.13</v>
+        <v>53.52</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>61.44</v>
+        <v>57.93</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>61.38</v>
+        <v>64.54000000000001</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1194,22 +1154,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>554.8</v>
+        <v>1144</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>54.59</v>
+        <v>53.02</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>38.49</v>
+        <v>45.94</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>38.05</v>
+        <v>39.84</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1218,22 +1178,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1029.85</v>
+        <v>1316.1</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>54.16</v>
+        <v>52.98</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>57.55</v>
+        <v>53.24</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>64.39</v>
+        <v>48.31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1242,22 +1202,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1946</v>
+        <v>3258</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>52.77</v>
+        <v>52.57</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>54.77</v>
+        <v>64.61</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>62.07</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1266,16 +1226,16 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1316</v>
+        <v>4045.8</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>52.27</v>
+        <v>52.39</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>46.01</v>
+        <v>53.45</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>47.6</v>
+        <v>57.75</v>
       </c>
     </row>
     <row r="19">
@@ -1290,22 +1250,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1420</v>
+        <v>1422.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>51.78</v>
+        <v>51.4</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>61.63</v>
+        <v>62.03</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>62</v>
+        <v>62.27</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1314,22 +1274,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1302.5</v>
+        <v>180.95</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>50.37</v>
+        <v>50.6</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>51.99</v>
+        <v>40.52</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>47.84</v>
+        <v>39.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1338,22 +1298,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1048.7</v>
+        <v>8800</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>49.43</v>
+        <v>50.43</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>53.62</v>
+        <v>64.7</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>61.55</v>
+        <v>67.90000000000001</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1362,22 +1322,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1477.1</v>
+        <v>1079.9</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>49.22</v>
+        <v>50.31</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>60.66</v>
+        <v>59.45</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>63</v>
+        <v>60.41</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1386,22 +1346,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>180.79</v>
+        <v>1047.5</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>48.78</v>
+        <v>49.39</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>40.37</v>
+        <v>53.43</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>39.87</v>
+        <v>61.49</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1410,22 +1370,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1584</v>
+        <v>548</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>48.62</v>
+        <v>49.39</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>58.21</v>
+        <v>37.15</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>56.29</v>
+        <v>37.09</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1434,22 +1394,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2302</v>
+        <v>186.5</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>48.3</v>
+        <v>48.77</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>45.16</v>
+        <v>46.68</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>38.09</v>
+        <v>57.28</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1458,22 +1418,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1245.8</v>
+        <v>1707.5</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>47.65</v>
+        <v>48.61</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>45.96</v>
+        <v>53.49</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>53.62</v>
+        <v>61.86</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1482,22 +1442,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1121</v>
+        <v>1913.3</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>47.14</v>
+        <v>47.73</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>43.54</v>
+        <v>58.88</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>38.78</v>
+        <v>61.35</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1506,22 +1466,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>11570</v>
+        <v>1086.9</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>45.96</v>
+        <v>47.53</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>50.85</v>
+        <v>59.46</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>54.14</v>
+        <v>69.91</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1530,22 +1490,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1432.2</v>
+        <v>3334</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>45.91</v>
+        <v>47.28</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>54.48</v>
+        <v>53.96</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>52.46</v>
+        <v>59.99</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1554,22 +1514,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>272.4</v>
+        <v>11589</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>45.89</v>
+        <v>47.2</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>41.39</v>
+        <v>51.14</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>50.01</v>
+        <v>54.28</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1578,22 +1538,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>244</v>
+        <v>5166</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>45.49</v>
+        <v>46.28</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>46.75</v>
+        <v>54.68</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>44.59</v>
+        <v>56.09</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1602,22 +1562,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>8693</v>
+        <v>1423.5</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>45.18</v>
+        <v>45.5</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>61.69</v>
+        <v>53.17</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>65.86</v>
+        <v>51.93</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1626,22 +1586,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2994.9</v>
+        <v>1178</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>45.15</v>
+        <v>44.88</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>62.28</v>
+        <v>42.43</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>58.33</v>
+        <v>47.61</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1650,22 +1610,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>5165</v>
+        <v>1454.6</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>45.01</v>
+        <v>43.89</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>53.47</v>
+        <v>57.3</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>55.4</v>
+        <v>61.46</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1674,22 +1634,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1700</v>
+        <v>1287</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>44.54</v>
+        <v>42.91</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>52.76</v>
+        <v>42.42</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>61.64</v>
+        <v>45.85</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1698,22 +1658,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>340</v>
+        <v>1014.1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>44.53</v>
+        <v>42.08</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>40.13</v>
+        <v>45.47</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>51.4</v>
+        <v>51.06</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1722,22 +1682,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1904</v>
+        <v>2898</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>43.5</v>
+        <v>41.59</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>57.24</v>
+        <v>46.06</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>60.43</v>
+        <v>41.59</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1746,22 +1706,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1174.7</v>
+        <v>1882.4</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>43.2</v>
+        <v>41.3</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>41.97</v>
+        <v>48.82</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>47.4</v>
+        <v>58.37</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1770,22 +1730,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>13565</v>
+        <v>238.4</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>42.76</v>
+        <v>39.76</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>48.18</v>
+        <v>43.65</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>52.87</v>
+        <v>43.58</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1794,22 +1754,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>2924</v>
+        <v>1773.2</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>42.33</v>
+        <v>39.27</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>46.84</v>
+        <v>42.98</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>41.78</v>
+        <v>51.13</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1818,22 +1778,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1792.9</v>
+        <v>266.05</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>40.46</v>
+        <v>39.06</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>45.29</v>
+        <v>38.19</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>52.62</v>
+        <v>48.45</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1842,22 +1802,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>183</v>
+        <v>1040.7</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>40.3</v>
+        <v>38.87</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>43.2</v>
+        <v>37.38</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>55.9</v>
+        <v>48.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1866,22 +1826,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1049</v>
+        <v>319.4</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>39.91</v>
+        <v>38.86</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>38.57</v>
+        <v>38.35</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>49.05</v>
+        <v>35.44</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1890,22 +1850,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>2640</v>
+        <v>720.3</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>39.6</v>
+        <v>38.45</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>52.56</v>
+        <v>34.53</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>51.68</v>
+        <v>39.77</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1914,16 +1874,16 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>236.4</v>
+        <v>13376</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>38.85</v>
+        <v>38.02</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>40.02</v>
+        <v>46.23</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>49.52</v>
+        <v>51.92</v>
       </c>
     </row>
     <row r="46">
@@ -1938,16 +1898,16 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>2028</v>
+        <v>2010.4</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>38.76</v>
+        <v>37.47</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>34.13</v>
+        <v>33.82</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>40.59</v>
+        <v>40.46</v>
       </c>
     </row>
     <row r="47">
@@ -1962,22 +1922,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>405.2</v>
+        <v>401</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>38.17</v>
+        <v>35.63</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>41.38</v>
+        <v>39.91</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>54.71</v>
+        <v>53.79</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1986,22 +1946,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>726.95</v>
+        <v>2608.7</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>37.81</v>
+        <v>35.13</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>35.58</v>
+        <v>50.4</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>40.24</v>
+        <v>50.95</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -2010,22 +1970,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>269.4</v>
+        <v>330.05</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>35.37</v>
+        <v>33.48</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>32.62</v>
+        <v>35.99</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>32.19</v>
+        <v>49.14</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -2034,22 +1994,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>317.9</v>
+        <v>266</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.17</v>
+        <v>32.82</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>37.79</v>
+        <v>31.25</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>35.36</v>
+        <v>31.69</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2058,16 +2018,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1000</v>
+        <v>232.25</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>32.56</v>
+        <v>32.63</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>43.53</v>
+        <v>38.13</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>50.34</v>
+        <v>48.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-09-05
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>5169.2</v>
+        <v>1325</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>71.93000000000001</v>
+        <v>58.41</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>73.76000000000001</v>
+        <v>62.84</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>69.19</v>
+        <v>66.7</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>50.87</v>
+        <v>31.12</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>4439.24</v>
+        <v>1242.55</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>4323.1</v>
+        <v>1221.95</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>811562</v>
+        <v>1627473</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>458669</v>
+        <v>323430</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>328</v>
+        <v>11919</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>65.69</v>
+        <v>57.18</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>68.17</v>
+        <v>75.04000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>66.01000000000001</v>
+        <v>67.83</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>41.27</v>
+        <v>51.63</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>280.96</v>
+        <v>10408.38</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>278.71</v>
+        <v>10157.2</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>31526889</v>
+        <v>259937</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>301937</v>
+        <v>327539</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1337.5</v>
+        <v>322.75</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>64.53</v>
+        <v>57.02</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>64.87</v>
+        <v>65.48</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>67.06999999999999</v>
+        <v>64.59</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>31.46</v>
+        <v>32.15</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1236.47</v>
+        <v>283.86</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1216.25</v>
+        <v>280.95</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1804528</v>
+        <v>36213900</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>325846</v>
+        <v>297104</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,37 +663,37 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11910</v>
+        <v>3310</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>64.43000000000001</v>
+        <v>55.68</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>74.95999999999999</v>
+        <v>65.91</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>68.81999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>52.36</v>
+        <v>23.43</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>10292.1</v>
+        <v>3040.43</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>10056.1</v>
+        <v>2989.23</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>341405</v>
+        <v>1016009</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>327022</v>
+        <v>225316</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -702,70 +702,31 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>8059</v>
+        <v>5027</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>60.94</v>
+        <v>53.1</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>64.83</v>
+        <v>66.66</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>69.45999999999999</v>
+        <v>66.98</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>35.22</v>
+        <v>41.21</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>7362.25</v>
+        <v>4471.74</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>7206.37</v>
+        <v>4352.64</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>436761</v>
+        <v>813457</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>221237</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>GRASIM</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>3258</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>52.57</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>64.61</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>67.8</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>25.33</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>3021.5</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>2972.27</v>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>880922</v>
-      </c>
-      <c r="K7" s="4" t="n">
-        <v>223145</v>
+        <v>445431</v>
       </c>
     </row>
   </sheetData>
@@ -775,7 +736,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -842,22 +802,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>423.7</v>
+        <v>421.15</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>74.16</v>
+        <v>66.53</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>61.93</v>
+        <v>62.18</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>56.77</v>
+        <v>56.97</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -866,22 +826,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>5169.2</v>
+        <v>415.35</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>71.93000000000001</v>
+        <v>62.17</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>73.76000000000001</v>
+        <v>49.06</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>69.19</v>
+        <v>57.43</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -890,22 +850,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>3168.5</v>
+        <v>1325</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>66.52</v>
+        <v>58.41</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>67.81</v>
+        <v>62.84</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>60.73</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -914,22 +874,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>328</v>
+        <v>11919</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>65.69</v>
+        <v>57.18</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>68.17</v>
+        <v>75.04000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>66.01000000000001</v>
+        <v>67.83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -938,22 +898,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1337.5</v>
+        <v>322.75</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>64.53</v>
+        <v>57.02</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>64.87</v>
+        <v>65.48</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>67.06999999999999</v>
+        <v>64.59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -962,22 +922,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>11910</v>
+        <v>188.79</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>64.43000000000001</v>
+        <v>56.03</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>74.95999999999999</v>
+        <v>48.88</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>68.81999999999999</v>
+        <v>57.82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -986,22 +946,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1640.9</v>
+        <v>3310</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>61.51</v>
+        <v>55.68</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>61.97</v>
+        <v>65.91</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>58.68</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1010,22 +970,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>8059</v>
+        <v>1322</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>60.94</v>
+        <v>55.16</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>64.83</v>
+        <v>47.73</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>69.45999999999999</v>
+        <v>48.34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1034,22 +994,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>411.9</v>
+        <v>1273</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>55.51</v>
+        <v>54.66</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>49.37</v>
+        <v>49.66</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>60.06</v>
+        <v>54.59</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1058,22 +1018,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1265</v>
+        <v>5027</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>54.95</v>
+        <v>53.1</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>48.57</v>
+        <v>66.66</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>54.58</v>
+        <v>66.98</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1082,22 +1042,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>2002</v>
+        <v>1707.3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>53.65</v>
+        <v>51.25</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>58.37</v>
+        <v>53.47</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>56.37</v>
+        <v>60.46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1106,22 +1066,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>2342</v>
+        <v>1992.1</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>53.64</v>
+        <v>50.76</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>47.46</v>
+        <v>55.59</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>38.69</v>
+        <v>54.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1130,22 +1090,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1037.4</v>
+        <v>546.4</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>53.52</v>
+        <v>50.41</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>57.93</v>
+        <v>36.83</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>64.54000000000001</v>
+        <v>37.17</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1154,22 +1114,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1144</v>
+        <v>1423.2</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>53.02</v>
+        <v>49.94</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>45.94</v>
+        <v>62.09</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>39.84</v>
+        <v>61.05</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1178,22 +1138,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1316.1</v>
+        <v>1596.9</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>52.98</v>
+        <v>49.52</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>53.24</v>
+        <v>57.65</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>48.31</v>
+        <v>56.71</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1202,22 +1162,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>3258</v>
+        <v>1130</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>52.57</v>
+        <v>49.14</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>64.61</v>
+        <v>44.69</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>67.8</v>
+        <v>39.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1226,22 +1186,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>4045.8</v>
+        <v>2304</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>52.39</v>
+        <v>48.19</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>53.45</v>
+        <v>45.51</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>57.75</v>
+        <v>38.32</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1250,22 +1210,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1422.8</v>
+        <v>1775</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>51.4</v>
+        <v>47.54</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>62.03</v>
+        <v>44.32</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>62.27</v>
+        <v>51.78</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1274,22 +1234,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>180.95</v>
+        <v>405.35</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>50.6</v>
+        <v>47.24</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>40.52</v>
+        <v>46.99</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>39.9</v>
+        <v>58.58</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1298,22 +1258,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>8800</v>
+        <v>1293.4</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>50.43</v>
+        <v>46.93</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>64.7</v>
+        <v>50.86</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>67.90000000000001</v>
+        <v>47.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1322,22 +1282,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1079.9</v>
+        <v>332.5</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>50.31</v>
+        <v>46.62</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>59.45</v>
+        <v>40.04</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>60.41</v>
+        <v>50.59</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1346,22 +1306,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1047.5</v>
+        <v>1010</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>49.39</v>
+        <v>46.26</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>53.43</v>
+        <v>53.89</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>61.49</v>
+        <v>63.24</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1370,22 +1330,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>548</v>
+        <v>1060.5</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>49.39</v>
+        <v>45.91</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>37.15</v>
+        <v>56.89</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>37.09</v>
+        <v>59.15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1394,22 +1354,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>186.5</v>
+        <v>1899</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>48.77</v>
+        <v>44.63</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>46.68</v>
+        <v>56.11</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>57.28</v>
+        <v>59.92</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1418,22 +1378,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1707.5</v>
+        <v>234.65</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>48.61</v>
+        <v>44.5</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>53.49</v>
+        <v>40.61</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>61.86</v>
+        <v>49.43</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1442,22 +1402,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1913.3</v>
+        <v>239.5</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>47.73</v>
+        <v>44.48</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>58.88</v>
+        <v>44.43</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>61.35</v>
+        <v>43.75</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1466,22 +1426,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1086.9</v>
+        <v>2938</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>47.53</v>
+        <v>43.68</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>59.46</v>
+        <v>55.94</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>69.91</v>
+        <v>56.89</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1490,22 +1450,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3334</v>
+        <v>3975</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>47.28</v>
+        <v>43.67</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>53.96</v>
+        <v>50.15</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>59.99</v>
+        <v>55.91</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1514,22 +1474,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>11589</v>
+        <v>8650</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>47.2</v>
+        <v>43.28</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>51.14</v>
+        <v>58.31</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>54.28</v>
+        <v>65.03</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1538,22 +1498,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>5166</v>
+        <v>176.4</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>46.28</v>
+        <v>43.08</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>54.68</v>
+        <v>37.59</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>56.09</v>
+        <v>38.93</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1562,16 +1522,16 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1423.5</v>
+        <v>266</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>45.5</v>
+        <v>41.63</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>53.17</v>
+        <v>38.16</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>51.93</v>
+        <v>48.52</v>
       </c>
     </row>
     <row r="33">
@@ -1586,22 +1546,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1178</v>
+        <v>1155</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>44.88</v>
+        <v>40.05</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>42.43</v>
+        <v>39.65</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>47.61</v>
+        <v>45.86</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1610,22 +1570,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1454.6</v>
+        <v>264.1</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>43.89</v>
+        <v>39.97</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>57.3</v>
+        <v>30.49</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>61.46</v>
+        <v>32.96</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1634,22 +1594,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1287</v>
+        <v>712.1</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>42.91</v>
+        <v>39.89</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>42.42</v>
+        <v>33.24</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>45.85</v>
+        <v>39.35</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1658,22 +1618,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1014.1</v>
+        <v>1840</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>42.08</v>
+        <v>39.89</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>45.47</v>
+        <v>45.29</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>51.06</v>
+        <v>55.92</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1682,22 +1642,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2898</v>
+        <v>1041</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>41.59</v>
+        <v>39.21</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>46.06</v>
+        <v>53.62</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>41.59</v>
+        <v>65.06999999999999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1706,22 +1666,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1882.4</v>
+        <v>1016.1</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>41.3</v>
+        <v>39.08</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>48.82</v>
+        <v>48.42</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>58.37</v>
+        <v>58.52</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1730,22 +1690,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>238.4</v>
+        <v>1416</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>39.76</v>
+        <v>38.45</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>43.65</v>
+        <v>51.31</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>43.58</v>
+        <v>58.25</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1754,22 +1714,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1773.2</v>
+        <v>984.8</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>39.27</v>
+        <v>37.42</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>42.98</v>
+        <v>42.22</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>51.13</v>
+        <v>49.38</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1778,22 +1738,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>266.05</v>
+        <v>4977</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>39.06</v>
+        <v>37.2</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>38.19</v>
+        <v>49.96</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>48.45</v>
+        <v>53.49</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1802,22 +1762,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1040.7</v>
+        <v>11275</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>38.87</v>
+        <v>36.88</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>37.38</v>
+        <v>48.21</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>48.5</v>
+        <v>52.93</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1826,22 +1786,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>319.4</v>
+        <v>1973.4</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>38.86</v>
+        <v>36.66</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>38.35</v>
+        <v>31.32</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>35.44</v>
+        <v>39.57</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1850,22 +1810,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>720.3</v>
+        <v>1385</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>38.45</v>
+        <v>36.22</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>34.53</v>
+        <v>47.69</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>39.77</v>
+        <v>49.59</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1874,22 +1834,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>13376</v>
+        <v>311.5</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>38.02</v>
+        <v>35.65</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46.23</v>
+        <v>36.5</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>51.92</v>
+        <v>35.17</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1898,22 +1858,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>2010.4</v>
+        <v>7630.5</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>37.47</v>
+        <v>35.18</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>33.82</v>
+        <v>53.98</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>40.46</v>
+        <v>64.45</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1922,22 +1882,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>401</v>
+        <v>1010</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>35.63</v>
+        <v>32.91</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>39.91</v>
+        <v>33.29</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>53.79</v>
+        <v>46.47</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1946,22 +1906,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>2608.7</v>
+        <v>2815.6</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>35.13</v>
+        <v>32.89</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>50.4</v>
+        <v>44.68</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>50.95</v>
+        <v>41.26</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1970,22 +1930,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>330.05</v>
+        <v>3150</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>33.48</v>
+        <v>32.01</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>35.99</v>
+        <v>46.74</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>49.14</v>
+        <v>55.51</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1994,22 +1954,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>266</v>
+        <v>2527.3</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>32.82</v>
+        <v>31.69</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>31.25</v>
+        <v>45.2</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>31.69</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -2018,16 +1978,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>232.25</v>
+        <v>12694</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>32.63</v>
+        <v>27.53</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>38.13</v>
+        <v>39.95</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>48.49</v>
+        <v>48.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-09-12
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -546,37 +546,37 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1325</v>
+        <v>323.5</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>58.41</v>
+        <v>57.58</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>62.84</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.7</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>31.12</v>
+        <v>24.69</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>1242.55</v>
+        <v>285.87</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>1221.95</v>
+        <v>282.75</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>1627473</v>
+        <v>31911776</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>323430</v>
+        <v>297794</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -585,37 +585,37 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>11919</v>
+        <v>3319</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>57.18</v>
+        <v>56.16</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>75.04000000000001</v>
+        <v>62.79</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>67.83</v>
+        <v>65.81</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>51.63</v>
+        <v>22.49</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>10408.38</v>
+        <v>3054.43</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>10157.2</v>
+        <v>3001.38</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>259937</v>
+        <v>1083968</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>327539</v>
+        <v>222596</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -624,37 +624,37 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>322.75</v>
+        <v>11768</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>57.02</v>
+        <v>51.88</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>65.48</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>64.59</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>32.15</v>
+        <v>44.63</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>283.86</v>
+        <v>10481.7</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>280.95</v>
+        <v>10224.97</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>36213900</v>
+        <v>231978</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>297104</v>
+        <v>320916</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -663,70 +663,31 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>3310</v>
+        <v>5009.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>55.68</v>
+        <v>51.21</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>65.91</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.3</v>
+        <v>66.77</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>23.43</v>
+        <v>28</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>3040.43</v>
+        <v>4512.96</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>2989.23</v>
+        <v>4391.36</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>1016009</v>
+        <v>737285</v>
       </c>
       <c r="K5" s="4" t="n">
-        <v>225316</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>5027</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>66.66</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>66.98</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>41.21</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>4471.74</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>4352.64</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>813457</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>445431</v>
+        <v>444499</v>
       </c>
     </row>
   </sheetData>
@@ -735,7 +696,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -793,7 +753,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -802,22 +762,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>421.15</v>
+        <v>426.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>66.53</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>62.18</v>
+        <v>53.42</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>56.97</v>
+        <v>59.26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -826,22 +786,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>415.35</v>
+        <v>419</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>62.17</v>
+        <v>59.87</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>49.06</v>
+        <v>59.27</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>57.43</v>
+        <v>55.94</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -850,22 +810,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1325</v>
+        <v>1764.6</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>58.41</v>
+        <v>58.67</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>62.84</v>
+        <v>59.12</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>66.7</v>
+        <v>62.01</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -874,22 +834,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11919</v>
+        <v>323.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>57.18</v>
+        <v>57.58</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>75.04000000000001</v>
+        <v>65.68000000000001</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>67.83</v>
+        <v>64.79000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -898,22 +858,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>322.75</v>
+        <v>3319</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>57.02</v>
+        <v>56.16</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>65.48</v>
+        <v>62.79</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>64.59</v>
+        <v>65.81</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -922,22 +882,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>188.79</v>
+        <v>8900</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>56.03</v>
+        <v>54.6</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>48.88</v>
+        <v>62.27</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>57.82</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -946,22 +906,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3310</v>
+        <v>3060</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>55.68</v>
+        <v>54.39</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>65.91</v>
+        <v>59.94</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>67.3</v>
+        <v>58.63</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -970,22 +930,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1322</v>
+        <v>1038.6</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>55.16</v>
+        <v>53.78</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>47.73</v>
+        <v>49.27</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>48.34</v>
+        <v>52.29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -994,16 +954,16 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1273</v>
+        <v>11768</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>54.66</v>
+        <v>51.88</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>49.66</v>
+        <v>69.04000000000001</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>54.59</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -1018,22 +978,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>5027</v>
+        <v>5009.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>53.1</v>
+        <v>51.21</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>66.66</v>
+        <v>66.18000000000001</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>66.98</v>
+        <v>66.77</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1042,22 +1002,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1707.3</v>
+        <v>1304</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>51.25</v>
+        <v>51.19</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>53.47</v>
+        <v>52.15</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>60.46</v>
+        <v>61.99</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1066,22 +1026,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1992.1</v>
+        <v>333.4</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>50.76</v>
+        <v>48.57</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>55.59</v>
+        <v>40.64</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>54.9</v>
+        <v>50.79</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1090,22 +1050,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>546.4</v>
+        <v>269.1</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>50.41</v>
+        <v>48.47</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>36.83</v>
+        <v>40.76</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>37.17</v>
+        <v>49.33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1114,22 +1074,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1423.2</v>
+        <v>1014</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>49.94</v>
+        <v>47.93</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>62.09</v>
+        <v>49.71</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>61.05</v>
+        <v>60.94</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1138,22 +1098,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1596.9</v>
+        <v>1165.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>49.52</v>
+        <v>47.78</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>57.65</v>
+        <v>41.86</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>56.71</v>
+        <v>46.86</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1162,22 +1122,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1130</v>
+        <v>1246</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>49.14</v>
+        <v>47.44</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>44.69</v>
+        <v>46.11</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>39.15</v>
+        <v>53.03</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1186,22 +1146,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2304</v>
+        <v>404.35</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>48.19</v>
+        <v>46.54</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>45.51</v>
+        <v>46.62</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>38.32</v>
+        <v>58.39</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1210,22 +1170,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1775</v>
+        <v>530</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>47.54</v>
+        <v>44.14</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>44.32</v>
+        <v>33.58</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>51.78</v>
+        <v>35.51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1234,22 +1194,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>405.35</v>
+        <v>708.25</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>47.24</v>
+        <v>43.99</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>46.99</v>
+        <v>32.62</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>58.58</v>
+        <v>38.95</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1258,22 +1218,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1293.4</v>
+        <v>183</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>46.93</v>
+        <v>43.84</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>50.86</v>
+        <v>43.94</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>47.48</v>
+        <v>55.86</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1282,22 +1242,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>332.5</v>
+        <v>232.5</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>46.62</v>
+        <v>42.59</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>40.04</v>
+        <v>39.52</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>50.59</v>
+        <v>48.85</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1306,22 +1266,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1010</v>
+        <v>1541</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>46.26</v>
+        <v>41.65</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>53.89</v>
+        <v>52.63</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>63.24</v>
+        <v>54.35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1330,22 +1290,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>1060.5</v>
+        <v>3930.7</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>45.91</v>
+        <v>41.18</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>56.89</v>
+        <v>48.82</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>59.15</v>
+        <v>55.18</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1354,22 +1314,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1899</v>
+        <v>1831.1</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>44.63</v>
+        <v>41.01</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>56.11</v>
+        <v>44.56</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>59.92</v>
+        <v>55.56</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1378,22 +1338,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>234.65</v>
+        <v>4973</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>44.5</v>
+        <v>38.78</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>40.61</v>
+        <v>49.87</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>49.43</v>
+        <v>53.44</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1402,22 +1362,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>239.5</v>
+        <v>2818.7</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>44.48</v>
+        <v>38.2</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>44.43</v>
+        <v>43.12</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>43.75</v>
+        <v>40.89</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1426,22 +1386,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>2938</v>
+        <v>1034.5</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>43.68</v>
+        <v>38.18</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>55.94</v>
+        <v>53.57</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>56.89</v>
+        <v>57.56</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1450,22 +1410,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3975</v>
+        <v>2200.8</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>43.67</v>
+        <v>38.18</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>50.15</v>
+        <v>40.62</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>55.91</v>
+        <v>36.77</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1474,22 +1434,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>8650</v>
+        <v>1028.6</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>43.28</v>
+        <v>37.92</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>58.31</v>
+        <v>52.12</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>65.03</v>
+        <v>64.15000000000001</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1498,22 +1458,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>176.4</v>
+        <v>1379.3</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>43.08</v>
+        <v>37.69</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>37.59</v>
+        <v>52.36</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>38.93</v>
+        <v>57.28</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1522,22 +1482,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>266</v>
+        <v>1861</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>41.63</v>
+        <v>37.53</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>38.16</v>
+        <v>49.14</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>48.52</v>
+        <v>56.87</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1546,22 +1506,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1155</v>
+        <v>1913.5</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>40.05</v>
+        <v>37.4</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>39.65</v>
+        <v>50.96</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>45.86</v>
+        <v>52.57</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1570,22 +1530,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>264.1</v>
+        <v>1257.5</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>39.97</v>
+        <v>37.11</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>30.49</v>
+        <v>40.34</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>32.96</v>
+        <v>44.16</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1594,22 +1554,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>712.1</v>
+        <v>1700.6</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>39.89</v>
+        <v>36.82</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>33.24</v>
+        <v>38.09</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>39.35</v>
+        <v>47.71</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1618,22 +1578,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1840</v>
+        <v>259.85</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>39.89</v>
+        <v>36.07</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>45.29</v>
+        <v>28.79</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>55.92</v>
+        <v>31.63</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1642,22 +1602,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1041</v>
+        <v>995.7</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>39.21</v>
+        <v>35.42</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>53.62</v>
+        <v>45.45</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>65.06999999999999</v>
+        <v>56.99</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1666,22 +1626,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1016.1</v>
+        <v>11000</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>39.08</v>
+        <v>34.74</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>48.42</v>
+        <v>42.31</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>58.52</v>
+        <v>49.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1690,22 +1650,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1416</v>
+        <v>229.9</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>38.45</v>
+        <v>34.07</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>51.31</v>
+        <v>39.31</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>58.25</v>
+        <v>41.98</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1714,22 +1674,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>984.8</v>
+        <v>1366</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>37.42</v>
+        <v>34.01</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>42.22</v>
+        <v>45.21</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>49.38</v>
+        <v>48.48</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1738,22 +1698,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>4977</v>
+        <v>7530</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>37.2</v>
+        <v>33.7</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>49.96</v>
+        <v>51.8</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>53.49</v>
+        <v>63.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1762,22 +1722,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>11275</v>
+        <v>1386.2</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>36.88</v>
+        <v>33.5</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>48.21</v>
+        <v>47.98</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>52.93</v>
+        <v>56.55</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1786,22 +1746,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1973.4</v>
+        <v>167.4</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>36.66</v>
+        <v>33.02</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>31.32</v>
+        <v>32.57</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>39.57</v>
+        <v>37.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1810,22 +1770,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1385</v>
+        <v>1206.1</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>36.22</v>
+        <v>32.98</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>47.69</v>
+        <v>42.93</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>49.59</v>
+        <v>44.48</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1834,22 +1794,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>311.5</v>
+        <v>1037.7</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>35.65</v>
+        <v>32.63</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>36.5</v>
+        <v>37.49</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>35.17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1858,22 +1818,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>7630.5</v>
+        <v>1927</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>35.18</v>
+        <v>30.77</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>53.98</v>
+        <v>28.47</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>64.45</v>
+        <v>38.21</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1882,22 +1842,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1010</v>
+        <v>3107</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>32.91</v>
+        <v>29.78</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>33.29</v>
+        <v>44.29</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>46.47</v>
+        <v>53.92</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1906,22 +1866,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>2815.6</v>
+        <v>991</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>32.89</v>
+        <v>29.21</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>44.68</v>
+        <v>31.03</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>41.26</v>
+        <v>45.28</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1930,16 +1890,16 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>3150</v>
+        <v>301.1</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>32.01</v>
+        <v>28.86</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>46.74</v>
+        <v>34.17</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>55.51</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="50">
@@ -1954,16 +1914,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>2527.3</v>
+        <v>2472.5</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>31.69</v>
+        <v>28.7</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>45.2</v>
+        <v>42.06</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>48.96</v>
+        <v>47.75</v>
       </c>
     </row>
     <row r="51">
@@ -1978,16 +1938,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>12694</v>
+        <v>12590</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>27.53</v>
+        <v>27.31</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>39.95</v>
+        <v>37.57</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>48.47</v>
+        <v>47.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-09-19
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -34,16 +34,16 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,18 +87,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -534,169 +548,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>ETERNAL</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>323.5</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>57.58</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>65.68000000000001</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>64.79000000000001</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>24.69</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>285.87</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>282.75</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>31911776</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>297794</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>GRASIM</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>3319</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>56.16</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>62.79</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>65.81</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>22.49</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>3054.43</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>3001.38</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>1083968</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>222596</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>11768</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>51.88</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>69.04000000000001</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>65.90000000000001</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>44.63</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>10481.7</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>10224.97</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>231978</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>320916</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TITAN</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>5009.5</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>51.21</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>66.18000000000001</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>66.77</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>4512.96</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>4391.36</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>737285</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>444499</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -753,7 +605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -762,22 +614,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>426.4</v>
+        <v>1824</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>65.90000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>53.42</v>
+        <v>64</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.26</v>
+        <v>63.49</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -786,22 +638,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>419</v>
+        <v>326.85</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>59.87</v>
+        <v>59.7</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>59.27</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>55.94</v>
+        <v>65.68000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -810,22 +662,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1764.6</v>
+        <v>1049.3</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>58.67</v>
+        <v>57.65</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>59.12</v>
+        <v>50.7</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>62.01</v>
+        <v>52.93</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -834,22 +686,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>323.5</v>
+        <v>731</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>57.58</v>
+        <v>56.03</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>65.68000000000001</v>
+        <v>39.77</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>64.79000000000001</v>
+        <v>41.39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -858,22 +710,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3319</v>
+        <v>416.5</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>56.16</v>
+        <v>55.57</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>62.79</v>
+        <v>55.93</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>65.81</v>
+        <v>54.43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -882,22 +734,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>8900</v>
+        <v>1185</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>54.6</v>
+        <v>55.28</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>62.27</v>
+        <v>44.78</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>67.8</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -906,22 +758,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>3060</v>
+        <v>550.95</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>54.39</v>
+        <v>55.23</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>59.94</v>
+        <v>40.76</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>58.63</v>
+        <v>37.87</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -930,22 +782,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1038.6</v>
+        <v>1893.3</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>53.78</v>
+        <v>54.4</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>49.27</v>
+        <v>50.55</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>52.29</v>
+        <v>57.99</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -954,22 +806,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>11768</v>
+        <v>418</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>51.88</v>
+        <v>53.77</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>69.04000000000001</v>
+        <v>46.95</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>65.90000000000001</v>
+        <v>56.47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -978,22 +830,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>5009.5</v>
+        <v>1766.9</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>51.21</v>
+        <v>53.73</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>66.18000000000001</v>
+        <v>42.55</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>66.77</v>
+        <v>49.77</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1002,22 +854,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1304</v>
+        <v>270.3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>51.19</v>
+        <v>52.24</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>52.15</v>
+        <v>41.77</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>61.99</v>
+        <v>49.64</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1026,22 +878,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>333.4</v>
+        <v>1257</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>48.57</v>
+        <v>52.14</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>40.64</v>
+        <v>47.75</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>50.79</v>
+        <v>53.65</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -1050,22 +902,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>269.1</v>
+        <v>185.54</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>48.47</v>
+        <v>49.69</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>40.76</v>
+        <v>46.49</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>49.33</v>
+        <v>56.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -1074,22 +926,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1014</v>
+        <v>8768.5</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>47.93</v>
+        <v>48.85</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>49.71</v>
+        <v>64.39</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>60.94</v>
+        <v>69.11</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1098,22 +950,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1165.5</v>
+        <v>1394.5</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>47.78</v>
+        <v>48.46</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>41.86</v>
+        <v>49.45</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>46.86</v>
+        <v>50.16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1122,22 +974,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1246</v>
+        <v>1275.6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>47.44</v>
+        <v>47.19</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>46.11</v>
+        <v>53.65</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>53.03</v>
+        <v>62.91</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1146,22 +998,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>404.35</v>
+        <v>1040.3</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>46.54</v>
+        <v>45.62</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>46.62</v>
+        <v>54.21</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>58.39</v>
+        <v>57.92</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1170,22 +1022,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>530</v>
+        <v>232.8</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>44.14</v>
+        <v>44.48</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>33.58</v>
+        <v>39.76</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>35.51</v>
+        <v>48.93</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1194,22 +1046,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>708.25</v>
+        <v>1249.3</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>43.99</v>
+        <v>44.27</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>32.62</v>
+        <v>47.31</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>38.95</v>
+        <v>45.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1218,22 +1070,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>183</v>
+        <v>1867.3</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>43.84</v>
+        <v>43.46</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>43.94</v>
+        <v>48.84</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>55.86</v>
+        <v>56.74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1242,22 +1094,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>232.5</v>
+        <v>262.3</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>42.59</v>
+        <v>43.43</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>39.52</v>
+        <v>31.17</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>48.85</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1266,22 +1118,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1541</v>
+        <v>1013.7</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>41.65</v>
+        <v>43.21</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>52.63</v>
+        <v>32.33</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>54.35</v>
+        <v>45.59</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1290,22 +1142,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>3930.7</v>
+        <v>2923.2</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>41.18</v>
+        <v>42.67</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>48.82</v>
+        <v>58.08</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>55.18</v>
+        <v>58.07</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1314,22 +1166,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1831.1</v>
+        <v>11014</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>41.01</v>
+        <v>42.57</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>44.56</v>
+        <v>42.57</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>55.56</v>
+        <v>50.04</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1338,46 +1190,46 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>4973</v>
+        <v>1537.1</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>38.78</v>
+        <v>42.41</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>49.87</v>
+        <v>52.29</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>53.44</v>
+        <v>54.19</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TRENT</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>2818.7</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>43.12</v>
-      </c>
-      <c r="F27" s="4" t="n">
-        <v>40.89</v>
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>11414</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>42.32</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>63.09</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>63.91</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1386,22 +1238,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>1034.5</v>
+        <v>996.2</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>38.18</v>
+        <v>41.86</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>53.57</v>
+        <v>45.53</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>57.56</v>
+        <v>57.03</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1410,22 +1262,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>2200.8</v>
+        <v>393.3</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>38.18</v>
+        <v>41.85</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>40.62</v>
+        <v>42.63</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>36.77</v>
+        <v>56.35</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1434,22 +1286,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>1028.6</v>
+        <v>3885</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>37.92</v>
+        <v>41.77</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>52.12</v>
+        <v>46.98</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>64.15000000000001</v>
+        <v>54.22</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1458,22 +1310,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>1379.3</v>
+        <v>303.8</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>37.69</v>
+        <v>40.56</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>52.36</v>
+        <v>35.33</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>57.28</v>
+        <v>34.64</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1482,22 +1334,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>1861</v>
+        <v>3187</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>37.53</v>
+        <v>40.31</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>49.14</v>
+        <v>57.48</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>56.87</v>
+        <v>63.27</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1506,22 +1358,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1913.5</v>
+        <v>2789</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>37.4</v>
+        <v>39.87</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>50.96</v>
+        <v>44.02</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>52.57</v>
+        <v>41.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1530,22 +1382,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1257.5</v>
+        <v>1010</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>37.11</v>
+        <v>39.72</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>40.34</v>
+        <v>49.88</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>44.16</v>
+        <v>62.82</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1554,22 +1406,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1700.6</v>
+        <v>229.89</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>36.82</v>
+        <v>39.44</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>38.09</v>
+        <v>39.31</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>47.71</v>
+        <v>41.98</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1578,22 +1430,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>259.85</v>
+        <v>972.7</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>36.07</v>
+        <v>39.28</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>28.79</v>
+        <v>50.41</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>31.63</v>
+        <v>61.32</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1602,22 +1454,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>995.7</v>
+        <v>1051.4</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>35.42</v>
+        <v>39.24</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>45.45</v>
+        <v>39.06</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>56.99</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1626,22 +1478,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>11000</v>
+        <v>1942.2</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>34.74</v>
+        <v>38.6</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>42.31</v>
+        <v>29.22</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>49.95</v>
+        <v>38.35</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1650,22 +1502,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>229.9</v>
+        <v>4845</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>34.07</v>
+        <v>37.16</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>39.31</v>
+        <v>48.51</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>41.98</v>
+        <v>52.81</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1674,16 +1526,16 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1366</v>
+        <v>323.65</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>34.01</v>
+        <v>36.31</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>45.21</v>
+        <v>36.35</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>48.48</v>
+        <v>48.51</v>
       </c>
     </row>
     <row r="41">
@@ -1698,22 +1550,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>7530</v>
+        <v>7516</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>33.7</v>
+        <v>36.01</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>51.8</v>
+        <v>51.48</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>63.2</v>
+        <v>63.03</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1722,22 +1574,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1386.2</v>
+        <v>166.83</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>33.5</v>
+        <v>35.53</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>47.98</v>
+        <v>32.28</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>56.55</v>
+        <v>36.99</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1746,22 +1598,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>167.4</v>
+        <v>1372.4</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>33.02</v>
+        <v>35.11</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>32.57</v>
+        <v>46.67</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>37.1</v>
+        <v>55.89</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1770,22 +1622,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>1206.1</v>
+        <v>4798.5</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>32.98</v>
+        <v>34.12</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>42.93</v>
+        <v>57.22</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>44.48</v>
+        <v>62.93</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1794,22 +1646,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1037.7</v>
+        <v>2451.3</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>32.63</v>
+        <v>33.92</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>37.49</v>
+        <v>40.88</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>36</v>
+        <v>47.3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1818,22 +1670,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>1927</v>
+        <v>2105</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>30.77</v>
+        <v>32.24</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>28.47</v>
+        <v>36.69</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>38.21</v>
+        <v>35.44</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1842,22 +1694,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>3107</v>
+        <v>1226.4</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>29.78</v>
+        <v>31.97</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>44.29</v>
+        <v>37.34</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>53.92</v>
+        <v>42.47</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1866,22 +1718,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>991</v>
+        <v>1852.5</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>29.21</v>
+        <v>31.51</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>31.03</v>
+        <v>46.47</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>45.28</v>
+        <v>50.27</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1890,22 +1742,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>301.1</v>
+        <v>3052</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>28.86</v>
+        <v>30.52</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>34.17</v>
+        <v>42.21</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>34.5</v>
+        <v>52.61</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1914,16 +1766,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>2472.5</v>
+        <v>1338.9</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>28.7</v>
+        <v>30.35</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>42.06</v>
+        <v>45.33</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>47.75</v>
+        <v>54.19</v>
       </c>
     </row>
     <row r="51">
@@ -1938,16 +1790,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>12590</v>
+        <v>12103</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>27.31</v>
+        <v>25.22</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>37.57</v>
+        <v>35.29</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>47.15</v>
+        <v>45.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-09-26
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -53,11 +53,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -87,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -99,15 +94,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -605,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -614,22 +600,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1824</v>
+        <v>335</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>64.3</v>
+        <v>61.08</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64</v>
+        <v>68.95999999999999</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>63.49</v>
+        <v>66.95999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -638,22 +624,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>326.85</v>
+        <v>1201</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>59.7</v>
+        <v>58.11</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>66.65000000000001</v>
+        <v>47.13</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>65.68000000000001</v>
+        <v>49.24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -662,22 +648,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1049.3</v>
+        <v>426.1</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>57.65</v>
+        <v>58.05</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>50.7</v>
+        <v>52.97</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>52.93</v>
+        <v>59.22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -686,22 +672,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>731</v>
+        <v>1785.3</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>56.03</v>
+        <v>56.52</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>39.77</v>
+        <v>59.37</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>41.39</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -710,22 +696,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>416.5</v>
+        <v>735.6</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>55.57</v>
+        <v>56.37</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>55.93</v>
+        <v>41.13</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>54.43</v>
+        <v>41.86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -734,22 +720,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1185</v>
+        <v>187.97</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>55.28</v>
+        <v>53.42</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>44.78</v>
+        <v>48.9</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>48.2</v>
+        <v>57.57</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -758,22 +744,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>550.95</v>
+        <v>269</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>55.23</v>
+        <v>52.77</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>40.76</v>
+        <v>37.35</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>37.87</v>
+        <v>34.42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -782,22 +768,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1893.3</v>
+        <v>8889</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>54.4</v>
+        <v>52.29</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>50.55</v>
+        <v>62.45</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>57.99</v>
+        <v>68.63</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -806,16 +792,16 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>418</v>
+        <v>269.5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>53.77</v>
+        <v>52.01</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>46.95</v>
+        <v>41.79</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>56.47</v>
+        <v>49.73</v>
       </c>
     </row>
     <row r="11">
@@ -830,22 +816,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1766.9</v>
+        <v>1755</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>53.73</v>
+        <v>51.58</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>42.55</v>
+        <v>43.59</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>49.77</v>
+        <v>50.28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -854,22 +840,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>270.3</v>
+        <v>1399.7</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>52.24</v>
+        <v>51.51</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>41.77</v>
+        <v>50.21</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>49.64</v>
+        <v>50.48</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -878,22 +864,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1257</v>
+        <v>235.86</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>52.14</v>
+        <v>49.99</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>47.75</v>
+        <v>42.3</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>53.65</v>
+        <v>49.75</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -902,22 +888,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>185.54</v>
+        <v>1277</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>49.69</v>
+        <v>48.58</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>46.49</v>
+        <v>53.85</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>56.8</v>
+        <v>63.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -926,22 +912,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>8768.5</v>
+        <v>1258</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>48.85</v>
+        <v>47.25</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>64.39</v>
+        <v>48.17</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>69.11</v>
+        <v>46.22</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -950,22 +936,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1394.5</v>
+        <v>4940</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>48.46</v>
+        <v>45.63</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>49.45</v>
+        <v>49.07</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>50.16</v>
+        <v>53.05</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -974,22 +960,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1275.6</v>
+        <v>1548</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>47.19</v>
+        <v>45.54</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>53.65</v>
+        <v>53.21</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>62.91</v>
+        <v>54.63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -998,22 +984,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1040.3</v>
+        <v>531</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>45.62</v>
+        <v>45.49</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>54.21</v>
+        <v>36.69</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>57.92</v>
+        <v>35.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1022,22 +1008,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>232.8</v>
+        <v>4884</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>44.48</v>
+        <v>45.46</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>39.76</v>
+        <v>59.6</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>48.93</v>
+        <v>64.43000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1046,22 +1032,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1249.3</v>
+        <v>11056</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>44.27</v>
+        <v>45.4</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>47.31</v>
+        <v>45.24</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>45.92</v>
+        <v>51.04</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1070,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1867.3</v>
+        <v>1222.4</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>43.46</v>
+        <v>44.66</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>48.84</v>
+        <v>43.29</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>56.74</v>
+        <v>51.74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1094,22 +1080,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>262.3</v>
+        <v>3876.2</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>43.43</v>
+        <v>43.86</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>31.17</v>
+        <v>46.62</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>32.4</v>
+        <v>54.04</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1118,22 +1104,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1013.7</v>
+        <v>1014</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>43.21</v>
+        <v>43.76</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>32.33</v>
+        <v>46.43</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>45.59</v>
+        <v>50.94</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1142,22 +1128,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>2923.2</v>
+        <v>977</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>42.67</v>
+        <v>43.64</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>58.08</v>
+        <v>49.01</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>58.07</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1166,22 +1152,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>11014</v>
+        <v>405</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>42.57</v>
+        <v>43.41</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>42.57</v>
+        <v>51.83</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>50.04</v>
+        <v>52.57</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1190,46 +1176,46 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1537.1</v>
+        <v>1849.9</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>42.41</v>
+        <v>43.2</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>52.29</v>
+        <v>50.62</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>54.19</v>
+        <v>57.48</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>11414</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>42.32</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>63.09</v>
-      </c>
-      <c r="F27" s="7" t="n">
-        <v>63.91</v>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>BEL</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>393.55</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>43.17</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>42.75</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>56.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1238,22 +1224,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>996.2</v>
+        <v>326.6</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>41.86</v>
+        <v>42.54</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>45.53</v>
+        <v>38.47</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>57.03</v>
+        <v>49.22</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1262,22 +1248,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>393.3</v>
+        <v>1942.9</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>41.85</v>
+        <v>42.47</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>42.63</v>
+        <v>30.91</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>56.35</v>
+        <v>38.64</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1286,22 +1272,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3885</v>
+        <v>3166.5</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>41.77</v>
+        <v>42.43</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>46.98</v>
+        <v>56.2</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>54.22</v>
+        <v>62.67</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1310,22 +1296,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>303.8</v>
+        <v>2900</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>40.56</v>
+        <v>41.92</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>35.33</v>
+        <v>53.46</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>34.64</v>
+        <v>56.57</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1334,22 +1320,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>3187</v>
+        <v>996.9</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>40.31</v>
+        <v>40.33</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>57.48</v>
+        <v>48.77</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>63.27</v>
+        <v>55.32</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1358,22 +1344,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>2789</v>
+        <v>983</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>39.87</v>
+        <v>39.59</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>44.02</v>
+        <v>43.53</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>41.05</v>
+        <v>56.08</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1382,22 +1368,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>1010</v>
+        <v>2444</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>39.72</v>
+        <v>39.55</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>49.88</v>
+        <v>40.45</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>62.82</v>
+        <v>47.14</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1406,22 +1392,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>229.89</v>
+        <v>1362.6</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>39.44</v>
+        <v>39.5</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>39.31</v>
+        <v>45.47</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>41.98</v>
+        <v>55.32</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1430,22 +1416,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>972.7</v>
+        <v>1785.4</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>39.28</v>
+        <v>38.15</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>50.41</v>
+        <v>42.06</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>61.32</v>
+        <v>53.41</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1454,22 +1440,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1051.4</v>
+        <v>1226</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>39.24</v>
+        <v>37.4</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>39.06</v>
+        <v>37.3</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>36.44</v>
+        <v>42.45</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1478,22 +1464,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>1942.2</v>
+        <v>11208</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>38.6</v>
+        <v>37.31</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>29.22</v>
+        <v>60.28</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>38.35</v>
+        <v>62.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1502,22 +1488,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>4845</v>
+        <v>227</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>37.16</v>
+        <v>36.78</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>48.51</v>
+        <v>37.79</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>52.81</v>
+        <v>41.47</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1526,22 +1512,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>323.65</v>
+        <v>983.2</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>36.31</v>
+        <v>36.53</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>36.35</v>
+        <v>30.73</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>48.51</v>
+        <v>44.81</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1550,22 +1536,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>7516</v>
+        <v>990</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>36.01</v>
+        <v>35.88</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>51.48</v>
+        <v>47.99</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>63.03</v>
+        <v>61.72</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1574,22 +1560,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>166.83</v>
+        <v>3035</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>35.53</v>
+        <v>35.06</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>32.28</v>
+        <v>41.55</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>36.99</v>
+        <v>52.22</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1598,22 +1584,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1372.4</v>
+        <v>164.02</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>35.11</v>
+        <v>33.97</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>46.67</v>
+        <v>30.8</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>55.89</v>
+        <v>36.45</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1622,22 +1608,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>4798.5</v>
+        <v>2082</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>34.12</v>
+        <v>32.02</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>57.22</v>
+        <v>35.79</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>62.93</v>
+        <v>35.13</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1646,22 +1632,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>2451.3</v>
+        <v>7360</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>33.92</v>
+        <v>31.88</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>40.88</v>
+        <v>48</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>47.3</v>
+        <v>61.19</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1670,22 +1656,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>2105</v>
+        <v>290.45</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>32.24</v>
+        <v>31.21</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>36.69</v>
+        <v>32.31</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>35.44</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1694,22 +1680,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>1226.4</v>
+        <v>12065</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>31.97</v>
+        <v>29.97</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>37.34</v>
+        <v>35</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>42.47</v>
+        <v>45.72</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1718,22 +1704,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1852.5</v>
+        <v>1000.2</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>31.51</v>
+        <v>29.92</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>46.47</v>
+        <v>35.48</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>50.27</v>
+        <v>34.86</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1742,16 +1728,16 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>3052</v>
+        <v>2669.3</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>30.52</v>
+        <v>29.67</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>42.21</v>
+        <v>39.23</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>52.61</v>
+        <v>39.93</v>
       </c>
     </row>
     <row r="50">
@@ -1766,22 +1752,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1338.9</v>
+        <v>1326.8</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>30.35</v>
+        <v>28.96</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>45.33</v>
+        <v>43.44</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>54.19</v>
+        <v>53.34</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1790,16 +1776,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>12103</v>
+        <v>1771</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>25.22</v>
+        <v>27.97</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>35.29</v>
+        <v>41.24</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>45.88</v>
+        <v>47.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-10-03
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -600,16 +600,16 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>335</v>
+        <v>418.35</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>61.08</v>
+        <v>57.56</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.95999999999999</v>
+        <v>57.5</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>66.95999999999999</v>
+        <v>55.74</v>
       </c>
     </row>
     <row r="3">
@@ -624,16 +624,16 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1201</v>
+        <v>1206.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>58.11</v>
+        <v>53.99</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>47.13</v>
+        <v>47.9</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>49.24</v>
+        <v>49.48</v>
       </c>
     </row>
     <row r="4">
@@ -648,22 +648,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>426.1</v>
+        <v>420.4</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>58.05</v>
+        <v>51.75</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>52.97</v>
+        <v>50.79</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>59.22</v>
+        <v>57.92</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -672,22 +672,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1785.3</v>
+        <v>721.2</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>56.52</v>
+        <v>49.31</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>59.37</v>
+        <v>38.22</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>62.6</v>
+        <v>40.46</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -696,22 +696,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>735.6</v>
+        <v>534.2</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>56.37</v>
+        <v>48.24</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>41.13</v>
+        <v>37.77</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>41.86</v>
+        <v>36.86</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -720,22 +720,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>187.97</v>
+        <v>1737.8</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>53.42</v>
+        <v>47.93</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>48.9</v>
+        <v>53.56</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>57.57</v>
+        <v>60.25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -744,22 +744,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>269</v>
+        <v>1721.6</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>52.77</v>
+        <v>46.56</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>37.35</v>
+        <v>42.07</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>34.42</v>
+        <v>49.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -768,22 +768,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>8889</v>
+        <v>4929.9</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>52.29</v>
+        <v>46.47</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>62.45</v>
+        <v>48.78</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>68.63</v>
+        <v>52.88</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -792,22 +792,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>269.5</v>
+        <v>1243.1</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>52.01</v>
+        <v>45.58</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>41.79</v>
+        <v>46.76</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>49.73</v>
+        <v>45.83</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -816,22 +816,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1755</v>
+        <v>1035</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>51.58</v>
+        <v>44.88</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>43.59</v>
+        <v>39.54</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>50.28</v>
+        <v>37.01</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -840,22 +840,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1399.7</v>
+        <v>1217.1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>51.51</v>
+        <v>44.52</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>50.21</v>
+        <v>42.63</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>50.48</v>
+        <v>51.43</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -864,22 +864,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>235.86</v>
+        <v>1533</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>49.99</v>
+        <v>44.2</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>42.3</v>
+        <v>51.73</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>49.75</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -888,22 +888,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1277</v>
+        <v>2816.8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>48.58</v>
+        <v>40.12</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>53.85</v>
+        <v>49.38</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>63.03</v>
+        <v>54.61</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -912,22 +912,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1258</v>
+        <v>313.9</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>47.25</v>
+        <v>39.24</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>48.17</v>
+        <v>57.83</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>46.22</v>
+        <v>62.24</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -936,22 +936,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>4940</v>
+        <v>1233</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>45.63</v>
+        <v>38.87</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>49.07</v>
+        <v>46.82</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>53.05</v>
+        <v>59.26</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -960,22 +960,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>1548</v>
+        <v>10710</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>45.54</v>
+        <v>37.99</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>53.21</v>
+        <v>39.07</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>54.63</v>
+        <v>47.91</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -984,22 +984,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>531</v>
+        <v>178</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>45.49</v>
+        <v>37.89</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>36.69</v>
+        <v>40.8</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>35.6</v>
+        <v>53.68</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1008,22 +1008,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>4884</v>
+        <v>1801</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>45.46</v>
+        <v>36.73</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>59.6</v>
+        <v>44.83</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>64.43000000000001</v>
+        <v>54.97</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1032,22 +1032,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>11056</v>
+        <v>383.1</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>45.4</v>
+        <v>36.41</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>45.24</v>
+        <v>39.08</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>51.04</v>
+        <v>54.53</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1056,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>1222.4</v>
+        <v>255.9</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>44.66</v>
+        <v>36.35</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>43.29</v>
+        <v>31.41</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>51.74</v>
+        <v>31.48</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1080,22 +1080,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>3876.2</v>
+        <v>2075</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>43.86</v>
+        <v>36.04</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>46.62</v>
+        <v>35.51</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>54.04</v>
+        <v>35.35</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1104,16 +1104,16 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>1014</v>
+        <v>2407</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>43.76</v>
+        <v>35.79</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>46.43</v>
+        <v>38.29</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>50.94</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="24">
@@ -1128,22 +1128,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>977</v>
+        <v>941.85</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>43.64</v>
+        <v>35.5</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>49.01</v>
+        <v>44.14</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>60.6</v>
+        <v>58.09</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1152,22 +1152,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>405</v>
+        <v>1344</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>43.41</v>
+        <v>34.76</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>51.83</v>
+        <v>42.82</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>52.57</v>
+        <v>47.24</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1176,22 +1176,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1849.9</v>
+        <v>254.55</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>43.2</v>
+        <v>34.73</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>50.62</v>
+        <v>33.46</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>57.48</v>
+        <v>45.86</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1200,22 +1200,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>393.55</v>
+        <v>1310.6</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>43.17</v>
+        <v>33.9</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>42.75</v>
+        <v>40.99</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>56.4</v>
+        <v>52.17</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1224,22 +1224,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>326.6</v>
+        <v>957</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>42.54</v>
+        <v>33.79</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>38.47</v>
+        <v>27.7</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>49.22</v>
+        <v>43.47</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1248,22 +1248,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1942.9</v>
+        <v>1741.1</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>42.47</v>
+        <v>32.36</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>30.91</v>
+        <v>39.15</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>38.64</v>
+        <v>51.26</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1272,22 +1272,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>3166.5</v>
+        <v>954.1</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>42.43</v>
+        <v>32.22</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>56.2</v>
+        <v>39.43</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>62.67</v>
+        <v>54.08</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1296,16 +1296,16 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>2900</v>
+        <v>159.35</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>41.92</v>
+        <v>32.19</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>53.46</v>
+        <v>28.47</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>56.57</v>
+        <v>35.74</v>
       </c>
     </row>
     <row r="32">
@@ -1320,22 +1320,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>996.9</v>
+        <v>948.3</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>40.33</v>
+        <v>32.06</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>48.77</v>
+        <v>43.51</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>55.32</v>
+        <v>52.62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1344,22 +1344,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>983</v>
+        <v>940.95</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>39.59</v>
+        <v>31.32</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>43.53</v>
+        <v>39.1</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>56.08</v>
+        <v>47.31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1368,22 +1368,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>2444</v>
+        <v>3693.4</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>39.55</v>
+        <v>31.26</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>40.45</v>
+        <v>39.75</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>47.14</v>
+        <v>50.45</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1392,22 +1392,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>1362.6</v>
+        <v>222.37</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>39.5</v>
+        <v>30.92</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>45.47</v>
+        <v>35.26</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>55.32</v>
+        <v>46.21</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1416,22 +1416,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1785.4</v>
+        <v>315.1</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>38.15</v>
+        <v>30.9</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>42.06</v>
+        <v>33.75</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>53.41</v>
+        <v>46.49</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1440,22 +1440,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1226</v>
+        <v>1307.7</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>37.4</v>
+        <v>30.13</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>37.3</v>
+        <v>39.36</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>42.45</v>
+        <v>52.29</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1464,22 +1464,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>11208</v>
+        <v>945</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>37.31</v>
+        <v>29.83</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>60.28</v>
+        <v>42.6</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>62.95</v>
+        <v>58.39</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1488,22 +1488,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>227</v>
+        <v>8133.5</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>36.78</v>
+        <v>29.69</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>37.79</v>
+        <v>43.34</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>41.47</v>
+        <v>58.37</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1512,22 +1512,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>983.2</v>
+        <v>1836</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>36.53</v>
+        <v>29.21</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>30.73</v>
+        <v>24.68</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>44.81</v>
+        <v>35.87</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1536,22 +1536,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>990</v>
+        <v>1167.7</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>35.88</v>
+        <v>27.92</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>47.99</v>
+        <v>32.11</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>61.72</v>
+        <v>39.55</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1560,22 +1560,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>3035</v>
+        <v>2962</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>35.06</v>
+        <v>27.86</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>41.55</v>
+        <v>43.15</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>52.22</v>
+        <v>55.75</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1584,22 +1584,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>164.02</v>
+        <v>279.4</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>33.97</v>
+        <v>27.34</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>30.8</v>
+        <v>30.02</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>36.45</v>
+        <v>33.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1608,22 +1608,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>2082</v>
+        <v>4515.7</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>32.02</v>
+        <v>26.52</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>35.79</v>
+        <v>47.35</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>35.13</v>
+        <v>58.34</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1632,22 +1632,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>7360</v>
+        <v>1732.6</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>31.88</v>
+        <v>24.8</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>48</v>
+        <v>39.01</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>61.19</v>
+        <v>46.31</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1656,22 +1656,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>290.45</v>
+        <v>2580</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>31.21</v>
+        <v>24.4</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>32.31</v>
+        <v>36.74</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>33.96</v>
+        <v>39.3</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1680,22 +1680,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>12065</v>
+        <v>2860</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>29.97</v>
+        <v>22.97</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>35</v>
+        <v>35.49</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>45.72</v>
+        <v>48.36</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1704,22 +1704,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1000.2</v>
+        <v>212.5</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>29.92</v>
+        <v>22.81</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>35.48</v>
+        <v>31.26</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>34.86</v>
+        <v>39.06</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1728,22 +1728,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>2669.3</v>
+        <v>11386</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>29.67</v>
+        <v>21.84</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>39.23</v>
+        <v>30.18</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>39.93</v>
+        <v>42.92</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1752,22 +1752,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>1326.8</v>
+        <v>10045</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>28.96</v>
+        <v>21.31</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>43.44</v>
+        <v>41.66</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>53.34</v>
+        <v>54.91</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1776,16 +1776,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>1771</v>
+        <v>6920</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>27.97</v>
+        <v>18.77</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>41.24</v>
+        <v>39.82</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>47.5</v>
+        <v>56.37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-10-10
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -34,13 +34,13 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="000563C1"/>
       <sz val="10"/>
+      <u val="single"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000563C1"/>
       <sz val="10"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -87,13 +87,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,49 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>441</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>67.95</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>64.59</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>59.85</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>33.54</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>402.04</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>401.48</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>19061203</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>438702</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -600,22 +642,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>418.35</v>
+        <v>441</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>57.56</v>
+        <v>67.95</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>57.5</v>
+        <v>64.59</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>55.74</v>
+        <v>59.85</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -624,22 +666,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1206.2</v>
+        <v>2918.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>53.99</v>
+        <v>61.06</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>47.9</v>
+        <v>49.74</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>49.48</v>
+        <v>42.78</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -648,22 +690,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>420.4</v>
+        <v>556.65</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>51.75</v>
+        <v>57.92</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>50.79</v>
+        <v>44.83</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>57.92</v>
+        <v>40.16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -672,22 +714,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>721.2</v>
+        <v>1259.1</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>49.31</v>
+        <v>55.97</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>38.22</v>
+        <v>49.21</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>40.46</v>
+        <v>53.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -696,22 +738,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>534.2</v>
+        <v>1761</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>48.24</v>
+        <v>50.94</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>37.77</v>
+        <v>55.72</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>36.86</v>
+        <v>61.22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -720,22 +762,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1737.8</v>
+        <v>1197</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>47.93</v>
+        <v>50.92</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>53.56</v>
+        <v>46.6</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>60.25</v>
+        <v>48.91</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -744,22 +786,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1721.6</v>
+        <v>2156</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>46.56</v>
+        <v>50.62</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>42.07</v>
+        <v>41.32</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>49.45</v>
+        <v>37.36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -768,22 +810,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>4929.9</v>
+        <v>266</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>46.47</v>
+        <v>50.46</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>48.78</v>
+        <v>39.41</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>52.88</v>
+        <v>33.61</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -792,22 +834,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1243.1</v>
+        <v>1355</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>45.58</v>
+        <v>49.53</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>46.76</v>
+        <v>49.42</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>45.83</v>
+        <v>55.08</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -816,22 +858,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1035</v>
+        <v>323.45</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>44.88</v>
+        <v>49.2</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>39.54</v>
+        <v>60.9</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>37.01</v>
+        <v>64.41</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -840,22 +882,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1217.1</v>
+        <v>1805.1</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>44.52</v>
+        <v>46.71</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>42.63</v>
+        <v>45.06</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>51.43</v>
+        <v>54.18</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -864,22 +906,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>1533</v>
+        <v>707.25</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>44.2</v>
+        <v>45.99</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>51.73</v>
+        <v>35.59</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>54</v>
+        <v>38.87</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -888,22 +930,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2816.8</v>
+        <v>411.55</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>40.12</v>
+        <v>45.35</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>49.38</v>
+        <v>47.51</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>54.61</v>
+        <v>55.88</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -912,22 +954,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>313.9</v>
+        <v>1023.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>39.24</v>
+        <v>45.3</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>57.83</v>
+        <v>38.66</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>62.24</v>
+        <v>36.37</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -936,22 +978,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1233</v>
+        <v>1216.7</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>38.87</v>
+        <v>44.45</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>46.82</v>
+        <v>44.28</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>59.26</v>
+        <v>44.79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -960,22 +1002,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>10710</v>
+        <v>162.57</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>37.99</v>
+        <v>43.63</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>39.07</v>
+        <v>32.28</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>47.91</v>
+        <v>36.83</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -984,22 +1026,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>178</v>
+        <v>1514.1</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>37.89</v>
+        <v>43.02</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>40.8</v>
+        <v>49.86</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>53.68</v>
+        <v>53.25</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1008,22 +1050,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1801</v>
+        <v>4833</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>36.73</v>
+        <v>42.2</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>44.83</v>
+        <v>45.97</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>54.97</v>
+        <v>51.68</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1032,22 +1074,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>383.1</v>
+        <v>1333</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>36.41</v>
+        <v>41.96</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>39.08</v>
+        <v>43.15</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>54.53</v>
+        <v>53.56</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1056,22 +1098,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>255.9</v>
+        <v>10675</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>36.35</v>
+        <v>41.82</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>31.41</v>
+        <v>38.62</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>31.48</v>
+        <v>47.67</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1080,22 +1122,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>2075</v>
+        <v>1684.6</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>36.04</v>
+        <v>41.7</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>35.51</v>
+        <v>39.38</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>35.35</v>
+        <v>47.66</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1104,22 +1146,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2407</v>
+        <v>959.1</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>35.79</v>
+        <v>39.88</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>38.29</v>
+        <v>40.48</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>46.4</v>
+        <v>54.43</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1128,22 +1170,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>941.85</v>
+        <v>3703.3</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>35.5</v>
+        <v>39.55</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>44.14</v>
+        <v>40.26</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>58.09</v>
+        <v>50.64</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1152,22 +1194,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1344</v>
+        <v>1856.7</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>34.76</v>
+        <v>38.7</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>42.82</v>
+        <v>27.72</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>47.24</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1176,22 +1218,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>254.55</v>
+        <v>7050</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>34.73</v>
+        <v>38.58</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>33.46</v>
+        <v>42.92</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>45.86</v>
+        <v>57.76</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1200,16 +1242,16 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>1310.6</v>
+        <v>960</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>33.9</v>
+        <v>37.63</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>40.99</v>
+        <v>45.04</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>52.17</v>
+        <v>53.28</v>
       </c>
     </row>
     <row r="28">
@@ -1224,22 +1266,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>33.79</v>
+        <v>37.53</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>27.7</v>
+        <v>27.48</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>43.47</v>
+        <v>43.32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1248,22 +1290,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>1741.1</v>
+        <v>8027.5</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>32.36</v>
+        <v>37.22</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>39.15</v>
+        <v>41.42</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>51.26</v>
+        <v>57.08</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1272,22 +1314,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>954.1</v>
+        <v>279.9</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>32.22</v>
+        <v>36.89</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>39.43</v>
+        <v>30.27</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>54.08</v>
+        <v>33.42</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1296,22 +1338,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>159.35</v>
+        <v>940.45</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>32.19</v>
+        <v>36.89</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>28.47</v>
+        <v>42.12</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>35.74</v>
+        <v>58.09</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1320,22 +1362,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>948.3</v>
+        <v>2339.1</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>32.06</v>
+        <v>35.81</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>43.51</v>
+        <v>34.64</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>52.62</v>
+        <v>44.95</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1344,22 +1386,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>940.95</v>
+        <v>214.62</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>31.32</v>
+        <v>35.66</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>39.1</v>
+        <v>33.08</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>47.31</v>
+        <v>39.41</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1368,22 +1410,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>3693.4</v>
+        <v>249.15</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>31.26</v>
+        <v>35.51</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>39.75</v>
+        <v>31.05</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>50.45</v>
+        <v>44.56</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1392,22 +1434,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>222.37</v>
+        <v>173.8</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>30.92</v>
+        <v>35.47</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>35.26</v>
+        <v>37.95</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>46.21</v>
+        <v>52.01</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1416,22 +1458,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>315.1</v>
+        <v>1170.3</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>30.9</v>
+        <v>35.42</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>33.75</v>
+        <v>32.56</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>46.49</v>
+        <v>39.67</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1440,22 +1482,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>1307.7</v>
+        <v>312</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>30.13</v>
+        <v>34.94</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>39.36</v>
+        <v>32.59</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>52.29</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1464,22 +1506,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>945</v>
+        <v>2634.4</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>29.83</v>
+        <v>34.21</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>42.6</v>
+        <v>42.93</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>58.39</v>
+        <v>51.23</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1488,22 +1530,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>8133.5</v>
+        <v>221.27</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>29.69</v>
+        <v>34.18</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>43.34</v>
+        <v>34.75</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>58.37</v>
+        <v>45.92</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1512,22 +1554,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1836</v>
+        <v>1760</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>29.21</v>
+        <v>33.66</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>24.68</v>
+        <v>40.8</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>35.87</v>
+        <v>53.02</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1536,22 +1578,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1167.7</v>
+        <v>1734.7</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>27.92</v>
+        <v>32.88</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>32.11</v>
+        <v>39.2</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>39.55</v>
+        <v>46.39</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1560,22 +1602,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>2962</v>
+        <v>11420</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>27.86</v>
+        <v>31.9</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>43.15</v>
+        <v>30.7</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>55.75</v>
+        <v>43.06</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1584,22 +1626,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>279.4</v>
+        <v>1168</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>27.34</v>
+        <v>31.05</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>30.02</v>
+        <v>38.76</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>33.4</v>
+        <v>54.26</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1608,22 +1650,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>4515.7</v>
+        <v>900.35</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>26.52</v>
+        <v>30.29</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>47.35</v>
+        <v>39.18</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>58.34</v>
+        <v>55.19</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1632,22 +1674,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1732.6</v>
+        <v>368.15</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>24.8</v>
+        <v>30.06</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>39.01</v>
+        <v>34.53</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>46.31</v>
+        <v>51.98</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1656,22 +1698,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>2580</v>
+        <v>4410</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>24.4</v>
+        <v>29.37</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>36.74</v>
+        <v>44.52</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>39.3</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1680,22 +1722,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2860</v>
+        <v>2890</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>22.97</v>
+        <v>28.28</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>35.49</v>
+        <v>40.01</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>48.36</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1704,22 +1746,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>212.5</v>
+        <v>883.8</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>22.81</v>
+        <v>27.75</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>31.26</v>
+        <v>34.51</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>39.06</v>
+        <v>44.48</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1728,22 +1770,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>11386</v>
+        <v>1301</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>21.84</v>
+        <v>26.85</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>30.18</v>
+        <v>38.14</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>42.92</v>
+        <v>44.86</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1752,22 +1794,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>10045</v>
+        <v>2796.2</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>21.31</v>
+        <v>25.77</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>41.66</v>
+        <v>33.57</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>54.91</v>
+        <v>47.05</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1776,16 +1818,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>6920</v>
+        <v>9778</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>18.77</v>
+        <v>23.2</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>39.82</v>
+        <v>38.87</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>56.37</v>
+        <v>53.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-10-17
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -546,31 +546,31 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>441</v>
+        <v>447.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>67.95</v>
+        <v>68.25</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64.59</v>
+        <v>66.3</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.85</v>
+        <v>60.88</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>33.54</v>
+        <v>39.12</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>402.04</v>
+        <v>404.71</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>401.48</v>
+        <v>403.62</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>19061203</v>
+        <v>20163344</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>438702</v>
+        <v>445068</v>
       </c>
     </row>
   </sheetData>
@@ -633,7 +633,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -642,22 +642,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>441</v>
+        <v>1790</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>67.95</v>
+        <v>75.58</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>64.59</v>
+        <v>68.04000000000001</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>59.85</v>
+        <v>61.74</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -666,22 +666,22 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2918.2</v>
+        <v>2465</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>61.06</v>
+        <v>74.02</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>49.74</v>
+        <v>57.66</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>42.78</v>
+        <v>44.22</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>WIPRO</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -690,22 +690,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>556.65</v>
+        <v>184.4</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>57.92</v>
+        <v>71.8</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>44.83</v>
+        <v>51.22</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>40.16</v>
+        <v>43.36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -714,22 +714,22 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1259.1</v>
+        <v>1380</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>55.97</v>
+        <v>70.16</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>49.21</v>
+        <v>59.61</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>53.64</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -738,22 +738,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1761</v>
+        <v>1161.2</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>50.94</v>
+        <v>69.83</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>55.72</v>
+        <v>52.18</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>61.22</v>
+        <v>43.26</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -762,22 +762,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1197</v>
+        <v>447.4</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>50.92</v>
+        <v>68.25</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>46.6</v>
+        <v>66.3</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>48.91</v>
+        <v>60.88</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -786,22 +786,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>2156</v>
+        <v>1290</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>50.62</v>
+        <v>62.8</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>41.32</v>
+        <v>53.44</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>37.36</v>
+        <v>55.13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>266</v>
+        <v>1905</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>50.46</v>
+        <v>61.87</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>39.41</v>
+        <v>52.77</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>33.61</v>
+        <v>58.06</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -834,22 +834,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1355</v>
+        <v>2958.7</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>49.53</v>
+        <v>61.73</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>49.42</v>
+        <v>51.03</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>55.08</v>
+        <v>43.19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -858,22 +858,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>323.45</v>
+        <v>1397</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>49.2</v>
+        <v>59.29</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>60.9</v>
+        <v>55.85</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>64.41</v>
+        <v>57.47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -882,22 +882,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1805.1</v>
+        <v>728.85</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>46.71</v>
+        <v>55.28</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>45.06</v>
+        <v>42.22</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>54.18</v>
+        <v>41.33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -906,22 +906,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>707.25</v>
+        <v>553</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>45.99</v>
+        <v>54.62</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>35.59</v>
+        <v>43.95</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>38.87</v>
+        <v>39.65</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>411.55</v>
+        <v>1218.8</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>45.35</v>
+        <v>54.59</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>47.51</v>
+        <v>52.09</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>55.88</v>
+        <v>51.21</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>INFY</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -954,22 +954,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1023.4</v>
+        <v>325.3</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>45.3</v>
+        <v>51.61</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>38.66</v>
+        <v>61.49</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>36.37</v>
+        <v>64.68000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1216.7</v>
+        <v>417.2</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>44.45</v>
+        <v>51.16</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>44.28</v>
+        <v>49.74</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>44.79</v>
+        <v>57.16</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>WIPRO</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -1002,22 +1002,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>162.57</v>
+        <v>263.5</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>43.63</v>
+        <v>49.17</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>32.28</v>
+        <v>38.22</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>36.83</v>
+        <v>32.79</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1026,22 +1026,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1514.1</v>
+        <v>1211.2</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>43.02</v>
+        <v>48.75</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>49.86</v>
+        <v>39.38</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>53.25</v>
+        <v>42.27</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1050,22 +1050,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>4833</v>
+        <v>1743.2</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>42.2</v>
+        <v>48.61</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>45.97</v>
+        <v>54.52</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>51.68</v>
+        <v>60.79</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1074,22 +1074,22 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1333</v>
+        <v>10862</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>41.96</v>
+        <v>48.5</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>43.15</v>
+        <v>43.25</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>53.56</v>
+        <v>49.29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>10675</v>
+        <v>978.9</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>41.82</v>
+        <v>47.64</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>38.62</v>
+        <v>34.27</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>47.67</v>
+        <v>45.1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1122,22 +1122,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1684.6</v>
+        <v>1893.8</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>41.7</v>
+        <v>47.49</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>39.38</v>
+        <v>32.94</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>47.66</v>
+        <v>37.65</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1146,22 +1146,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>959.1</v>
+        <v>7225</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>39.88</v>
+        <v>47.48</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>40.48</v>
+        <v>48.1</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>54.43</v>
+        <v>59.92</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>3703.3</v>
+        <v>982.1</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>39.55</v>
+        <v>47.29</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>40.26</v>
+        <v>47.93</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>50.64</v>
+        <v>54.36</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1194,22 +1194,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>1856.7</v>
+        <v>2920.9</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>38.7</v>
+        <v>46.3</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>27.72</v>
+        <v>40.37</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>36.4</v>
+        <v>49.68</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1218,22 +1218,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>7050</v>
+        <v>1216.3</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>38.58</v>
+        <v>45.26</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>42.92</v>
+        <v>46.17</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>57.76</v>
+        <v>57.89</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1242,22 +1242,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>960</v>
+        <v>962.6</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>37.63</v>
+        <v>44.71</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>45.04</v>
+        <v>41.24</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>53.28</v>
+        <v>54.65</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TATACONSUM</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1266,22 +1266,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>955</v>
+        <v>286.85</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>37.53</v>
+        <v>44.29</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>27.48</v>
+        <v>33.68</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>43.32</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1290,13 +1290,13 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>8027.5</v>
+        <v>10405</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>37.22</v>
+        <v>42.81</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>41.42</v>
+        <v>47.73</v>
       </c>
       <c r="F29" s="4" t="n">
         <v>57.08</v>
@@ -1305,7 +1305,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1314,22 +1314,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>279.9</v>
+        <v>315.15</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>36.89</v>
+        <v>41.6</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>30.27</v>
+        <v>35.03</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>33.42</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1338,22 +1338,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>940.45</v>
+        <v>175.5</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>36.89</v>
+        <v>41.33</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>42.12</v>
+        <v>39.78</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>58.09</v>
+        <v>52.67</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1362,22 +1362,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>2339.1</v>
+        <v>939.95</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>35.81</v>
+        <v>41.21</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>34.64</v>
+        <v>42.07</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>44.95</v>
+        <v>58.06</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1386,22 +1386,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>214.62</v>
+        <v>1328</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>35.66</v>
+        <v>41.09</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>33.08</v>
+        <v>41.97</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>39.41</v>
+        <v>46.17</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1410,22 +1410,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>249.15</v>
+        <v>376.85</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>35.51</v>
+        <v>40.75</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>31.05</v>
+        <v>38.98</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>44.56</v>
+        <v>53.43</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1434,22 +1434,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>173.8</v>
+        <v>908</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>35.47</v>
+        <v>40.3</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>37.95</v>
+        <v>40.51</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>52.01</v>
+        <v>55.7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1458,22 +1458,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>1170.3</v>
+        <v>216.25</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>35.42</v>
+        <v>40.29</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>32.56</v>
+        <v>34.52</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>39.67</v>
+        <v>39.69</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1482,22 +1482,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>312</v>
+        <v>2700</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>34.94</v>
+        <v>40.22</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>32.59</v>
+        <v>45.36</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>45.8</v>
+        <v>52.25</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1506,22 +1506,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>2634.4</v>
+        <v>222</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>34.21</v>
+        <v>39.28</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>42.93</v>
+        <v>35.42</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>51.23</v>
+        <v>46.11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>221.27</v>
+        <v>1656.8</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>34.18</v>
+        <v>38.97</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>34.75</v>
+        <v>37.45</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>45.92</v>
+        <v>46.42</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1554,22 +1554,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>1760</v>
+        <v>250.45</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>33.66</v>
+        <v>38.81</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>40.8</v>
+        <v>32.31</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>53.02</v>
+        <v>44.87</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1578,22 +1578,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1734.7</v>
+        <v>2331.9</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>32.88</v>
+        <v>37.91</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>39.2</v>
+        <v>34.27</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>46.39</v>
+        <v>44.8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1602,22 +1602,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>11420</v>
+        <v>1764</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>31.9</v>
+        <v>37.87</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>30.7</v>
+        <v>40.68</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>43.06</v>
+        <v>52.96</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1626,22 +1626,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>1168</v>
+        <v>11445</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>31.05</v>
+        <v>37.49</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>38.76</v>
+        <v>31.8</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>54.26</v>
+        <v>43.33</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1650,22 +1650,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>900.35</v>
+        <v>7890</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>30.29</v>
+        <v>37.32</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>39.18</v>
+        <v>39.02</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>55.19</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1674,22 +1674,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>368.15</v>
+        <v>1729</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>30.06</v>
+        <v>37.15</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>34.53</v>
+        <v>38.84</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>51.98</v>
+        <v>46.18</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1698,22 +1698,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>4410</v>
+        <v>4686.9</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>29.37</v>
+        <v>37.03</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>44.52</v>
+        <v>42.04</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>56.7</v>
+        <v>49.98</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1722,22 +1722,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>2890</v>
+        <v>3627.1</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>28.28</v>
+        <v>36.79</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>40.01</v>
+        <v>37.6</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>53.8</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MAXHEALTH</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1746,22 +1746,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>883.8</v>
+        <v>1265.5</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>27.75</v>
+        <v>35.77</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>34.51</v>
+        <v>36.58</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>44.48</v>
+        <v>50.03</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1770,22 +1770,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>1301</v>
+        <v>4444.8</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>26.85</v>
+        <v>35.04</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>38.14</v>
+        <v>45.67</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>44.86</v>
+        <v>57.23</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1794,22 +1794,22 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>2796.2</v>
+        <v>2885.9</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>25.77</v>
+        <v>33.19</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>33.57</v>
+        <v>41.91</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>47.05</v>
+        <v>54.6</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>MAXHEALTH</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -1818,16 +1818,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>9778</v>
+        <v>846</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>23.2</v>
+        <v>24.5</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>38.87</v>
+        <v>31.85</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>53.4</v>
+        <v>42.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Weekly RSI Screener Report – 2026-10-24
</commit_message>
<xml_diff>
--- a/docs/Nifty50_stocks.xlsx
+++ b/docs/Nifty50_stocks.xlsx
@@ -34,13 +34,13 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -87,13 +87,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -534,49 +534,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>KOTAKBANK</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n">
-        <v>447.4</v>
-      </c>
-      <c r="D2" s="4" t="n">
-        <v>68.25</v>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>66.3</v>
-      </c>
-      <c r="F2" s="4" t="n">
-        <v>60.88</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>39.12</v>
-      </c>
-      <c r="H2" s="4" t="n">
-        <v>404.71</v>
-      </c>
-      <c r="I2" s="4" t="n">
-        <v>403.62</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>20163344</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>445068</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -633,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>TCS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -642,22 +600,22 @@
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>1790</v>
+        <v>2530</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>75.58</v>
+        <v>74.67</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>68.04000000000001</v>
+        <v>60.09</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>61.74</v>
+        <v>45.43</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TCS</t>
+          <t>HCLTECH</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -666,16 +624,16 @@
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>2465</v>
+        <v>1422.2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>74.02</v>
+        <v>73.67</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>57.66</v>
+        <v>62.31</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>44.22</v>
+        <v>52.91</v>
       </c>
     </row>
     <row r="4">
@@ -690,22 +648,22 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>184.4</v>
+        <v>189.84</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>71.8</v>
+        <v>72.62</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>51.22</v>
+        <v>54.62</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>43.36</v>
+        <v>44.78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HCLTECH</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -714,16 +672,16 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1380</v>
+        <v>1790</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>70.16</v>
+        <v>71.66</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>59.61</v>
+        <v>68.69</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>51.5</v>
+        <v>62.11</v>
       </c>
     </row>
     <row r="6">
@@ -738,22 +696,22 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1161.2</v>
+        <v>1153.8</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>69.83</v>
+        <v>63.84</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>52.18</v>
+        <v>51.53</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>43.26</v>
+        <v>42.93</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -762,22 +720,22 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>447.4</v>
+        <v>1892.1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>68.25</v>
+        <v>58.67</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>66.3</v>
+        <v>51.76</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>60.88</v>
+        <v>57.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>AXISBANK</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -786,22 +744,22 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1290</v>
+        <v>1394.2</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>62.8</v>
+        <v>57.41</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>53.44</v>
+        <v>55.35</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>55.13</v>
+        <v>57.32</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>DRREDDY</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -810,22 +768,22 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1905</v>
+        <v>1229.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>61.87</v>
+        <v>55.21</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>52.77</v>
+        <v>51.54</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>58.06</v>
+        <v>50.98</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TRENT</t>
+          <t>KOTAKBANK</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -834,22 +792,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>2958.7</v>
+        <v>430.5</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>61.73</v>
+        <v>51.74</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>51.03</v>
+        <v>58.29</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>43.19</v>
+        <v>58.04</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -858,22 +816,22 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1397</v>
+        <v>10958</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>59.29</v>
+        <v>51.67</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>55.85</v>
+        <v>45.96</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>57.47</v>
+        <v>50.34</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -882,22 +840,22 @@
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>728.85</v>
+        <v>227.5</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>55.28</v>
+        <v>50.21</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>42.22</v>
+        <v>40.35</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>41.33</v>
+        <v>47.61</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HDFCLIFE</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -906,22 +864,22 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>553</v>
+        <v>317.4</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>54.62</v>
+        <v>47.44</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>43.95</v>
+        <v>57.53</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>39.65</v>
+        <v>63.17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>DRREDDY</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -930,22 +888,22 @@
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1218.8</v>
+        <v>1338</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>54.59</v>
+        <v>46.88</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>52.09</v>
+        <v>43.96</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>51.21</v>
+        <v>46.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -954,22 +912,22 @@
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>325.3</v>
+        <v>1190</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>51.61</v>
+        <v>44.35</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>61.49</v>
+        <v>37.28</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>64.68000000000001</v>
+        <v>40.73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>COALINDIA</t>
+          <t>SBIN</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -978,16 +936,16 @@
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>417.2</v>
+        <v>958.6</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>51.16</v>
+        <v>44.15</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>49.74</v>
+        <v>40.6</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>57.16</v>
+        <v>54.4</v>
       </c>
     </row>
     <row r="17">
@@ -1002,22 +960,22 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>263.5</v>
+        <v>257.9</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>49.17</v>
+        <v>43.96</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>38.22</v>
+        <v>35.63</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>32.79</v>
+        <v>31.78</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>AXISBANK</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1026,22 +984,22 @@
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>1211.2</v>
+        <v>1217.5</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>48.75</v>
+        <v>43.38</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>39.38</v>
+        <v>44.15</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>42.27</v>
+        <v>51.45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1050,22 +1008,22 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1743.2</v>
+        <v>7084.5</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>48.61</v>
+        <v>42.55</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>54.52</v>
+        <v>44.08</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>60.79</v>
+        <v>57.94</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1074,16 +1032,16 @@
         </is>
       </c>
       <c r="C20" s="4" t="n">
-        <v>10862</v>
+        <v>1702.7</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>48.5</v>
+        <v>42.52</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>43.25</v>
+        <v>49.15</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>49.29</v>
+        <v>58.83</v>
       </c>
     </row>
     <row r="21">
@@ -1098,22 +1056,22 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>978.9</v>
+        <v>959.8</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>47.64</v>
+        <v>41.84</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>34.27</v>
+        <v>32.23</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>45.1</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>HINDUNILVR</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1122,22 +1080,22 @@
         </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1893.8</v>
+        <v>2861.2</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>47.49</v>
+        <v>41.1</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>32.94</v>
+        <v>38.35</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>37.65</v>
+        <v>48.38</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>HDFCBANK</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1146,22 +1104,22 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>7225</v>
+        <v>692.8</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>47.48</v>
+        <v>40.86</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>48.1</v>
+        <v>35.63</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>59.92</v>
+        <v>37.78</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>BAJFINANCE</t>
+          <t>TRENT</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1170,22 +1128,22 @@
         </is>
       </c>
       <c r="C24" s="4" t="n">
-        <v>982.1</v>
+        <v>2727.5</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>47.29</v>
+        <v>40.55</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>47.93</v>
+        <v>44.04</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>54.36</v>
+        <v>40.78</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>HDFCLIFE</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1194,22 +1152,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2920.9</v>
+        <v>523.75</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>46.3</v>
+        <v>40.51</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>40.37</v>
+        <v>37.63</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>49.68</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>JSWSTEEL</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1218,22 +1176,22 @@
         </is>
       </c>
       <c r="C26" s="4" t="n">
-        <v>1216.3</v>
+        <v>3647</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>45.26</v>
+        <v>40.06</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>46.17</v>
+        <v>38.74</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>57.89</v>
+        <v>49.57</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>JSWSTEEL</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1242,22 +1200,22 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>962.6</v>
+        <v>1185.5</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>44.71</v>
+        <v>39.7</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>41.24</v>
+        <v>42.63</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>54.65</v>
+        <v>55.52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>TMPV</t>
+          <t>BAJFINANCE</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1266,22 +1224,22 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>286.85</v>
+        <v>928.95</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>44.29</v>
+        <v>37.99</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>33.68</v>
+        <v>42.19</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>33.96</v>
+        <v>51.57</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BAJAJ-AUTO</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1290,22 +1248,22 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>10405</v>
+        <v>1640</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>42.81</v>
+        <v>37.47</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>47.73</v>
+        <v>36.29</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>57.08</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>NTPC</t>
+          <t>BAJAJ-AUTO</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1314,22 +1272,22 @@
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>315.15</v>
+        <v>10072</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>41.6</v>
+        <v>37.32</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>35.03</v>
+        <v>44.07</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>46.5</v>
+        <v>55.07</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>TATASTEEL</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1338,22 +1296,22 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>175.5</v>
+        <v>2307</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>41.33</v>
+        <v>37.21</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>39.78</v>
+        <v>32.94</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>52.67</v>
+        <v>44.3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1362,22 +1320,22 @@
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>939.95</v>
+        <v>1748</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>41.21</v>
+        <v>37.16</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>42.07</v>
+        <v>39.6</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>58.06</v>
+        <v>52.47</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>GRASIM</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1386,22 +1344,22 @@
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1328</v>
+        <v>2894</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>41.09</v>
+        <v>36.71</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>41.97</v>
+        <v>40.7</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>46.17</v>
+        <v>53.91</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BEL</t>
+          <t>COALINDIA</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1410,22 +1368,22 @@
         </is>
       </c>
       <c r="C34" s="4" t="n">
-        <v>376.85</v>
+        <v>397.45</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>40.75</v>
+        <v>36.63</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>38.98</v>
+        <v>42.89</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>53.43</v>
+        <v>52.91</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>HINDALCO</t>
+          <t>HINDUNILVR</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1434,22 +1392,22 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>908</v>
+        <v>1814.7</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>40.3</v>
+        <v>36.39</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>40.51</v>
+        <v>28.25</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>55.7</v>
+        <v>35.35</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>POWERGRID</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1458,22 +1416,22 @@
         </is>
       </c>
       <c r="C36" s="4" t="n">
-        <v>216.25</v>
+        <v>247.4</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>40.29</v>
+        <v>36.31</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>34.52</v>
+        <v>30.88</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>39.69</v>
+        <v>44.15</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ADANIENT</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1482,22 +1440,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>2700</v>
+        <v>11230</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>40.22</v>
+        <v>34.96</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>45.36</v>
+        <v>29.88</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>52.25</v>
+        <v>42.32</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1506,22 +1464,22 @@
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>222</v>
+        <v>869.85</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>39.28</v>
+        <v>32.29</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>35.42</v>
+        <v>36.26</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>46.11</v>
+        <v>53.24</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>SBILIFE</t>
+          <t>ADANIENT</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1530,22 +1488,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1656.8</v>
+        <v>2550</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>38.97</v>
+        <v>32.14</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>37.45</v>
+        <v>38.74</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>46.42</v>
+        <v>48.63</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>POWERGRID</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1554,22 +1512,22 @@
         </is>
       </c>
       <c r="C40" s="4" t="n">
-        <v>250.45</v>
+        <v>7604.5</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>38.81</v>
+        <v>31.49</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>32.31</v>
+        <v>36.37</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>44.87</v>
+        <v>53.76</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1578,22 +1536,22 @@
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>2331.9</v>
+        <v>4549</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>37.91</v>
+        <v>31.43</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>34.27</v>
+        <v>38.68</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>44.8</v>
+        <v>48.47</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>SUNPHARMA</t>
+          <t>BEL</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1602,22 +1560,22 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>1764</v>
+        <v>362</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>37.87</v>
+        <v>31.17</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>40.68</v>
+        <v>34.65</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>52.96</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TATASTEEL</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1626,22 +1584,22 @@
         </is>
       </c>
       <c r="C43" s="4" t="n">
-        <v>11445</v>
+        <v>167.67</v>
       </c>
       <c r="D43" s="4" t="n">
-        <v>37.49</v>
+        <v>30.79</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>31.8</v>
+        <v>34.7</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>43.33</v>
+        <v>49.74</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -1650,22 +1608,22 @@
         </is>
       </c>
       <c r="C44" s="4" t="n">
-        <v>7890</v>
+        <v>865</v>
       </c>
       <c r="D44" s="4" t="n">
-        <v>37.32</v>
+        <v>30.16</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>39.02</v>
+        <v>34.72</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>55.5</v>
+        <v>53.59</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BAJAJFINSV</t>
+          <t>TMPV</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -1674,22 +1632,22 @@
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>1729</v>
+        <v>264.6</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>37.15</v>
+        <v>29.74</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>38.84</v>
+        <v>28.82</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>46.18</v>
+        <v>32.64</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>JIOFIN</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -1698,22 +1656,22 @@
         </is>
       </c>
       <c r="C46" s="4" t="n">
-        <v>4686.9</v>
+        <v>205.03</v>
       </c>
       <c r="D46" s="4" t="n">
-        <v>37.03</v>
+        <v>28.8</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>42.04</v>
+        <v>29.78</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>49.98</v>
+        <v>37.87</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>TITAN</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -1722,22 +1680,22 @@
         </is>
       </c>
       <c r="C47" s="4" t="n">
-        <v>3627.1</v>
+        <v>4299.7</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>36.79</v>
+        <v>28.05</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>37.6</v>
+        <v>41.78</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>49.2</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>NESTLEIND</t>
+          <t>BAJAJFINSV</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -1746,22 +1704,22 @@
         </is>
       </c>
       <c r="C48" s="4" t="n">
-        <v>1265.5</v>
+        <v>1655</v>
       </c>
       <c r="D48" s="4" t="n">
-        <v>35.77</v>
+        <v>27.89</v>
       </c>
       <c r="E48" s="4" t="n">
-        <v>36.58</v>
+        <v>34.42</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>50.03</v>
+        <v>43.88</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -1770,22 +1728,22 @@
         </is>
       </c>
       <c r="C49" s="4" t="n">
-        <v>4444.8</v>
+        <v>298</v>
       </c>
       <c r="D49" s="4" t="n">
-        <v>35.04</v>
+        <v>26.69</v>
       </c>
       <c r="E49" s="4" t="n">
-        <v>45.67</v>
+        <v>28.89</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>57.23</v>
+        <v>42.89</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GRASIM</t>
+          <t>NESTLEIND</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -1794,16 +1752,16 @@
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>2885.9</v>
+        <v>1175</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>33.19</v>
+        <v>26.69</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>41.91</v>
+        <v>29.99</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>54.6</v>
+        <v>45.78</v>
       </c>
     </row>
     <row r="51">
@@ -1818,16 +1776,16 @@
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>846</v>
+        <v>815</v>
       </c>
       <c r="D51" s="4" t="n">
-        <v>24.5</v>
+        <v>20.81</v>
       </c>
       <c r="E51" s="4" t="n">
-        <v>31.85</v>
+        <v>29.82</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>42.83</v>
+        <v>41.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>